<commit_message>
chore: align project docs with v3 baseline
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tien_Day_Professional_Build_Plan.xlsx
+++ b/Tien_Day_Professional_Build_Plan.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>index_v3.html — prototype đã chốt</t>
+          <t>Demo/ is the current V3 UX/UI source of truth. When documentation conflicts with Demo/, Demo/ wins until explicitly changed.</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,10 @@
           <t>Tiền Đây không cần nhiều hơn. Nó cần nhẹ hơn.
 Home chỉ ưu tiên chi tiêu + giao dịch + nút +.
 Lương / ngân sách / tiết kiệm nằm trong khu vực Tài chính riêng.
-GITHUB/GIT: CHỈ 1 REPOSITORY DUY NHẤT CHO TOÀN BỘ DỰ ÁN. Không tạo repo mới, không tạo project duplicate.</t>
+GITHUB/GIT: CHỈ 1 REPOSITORY DUY NHẤT CHO TOÀN BỘ DỰ ÁN. Không tạo repo mới, không tạo project duplicate.
+Demo/ is the current V3 UX/UI source of truth. When documentation conflicts with Demo/, Demo/ wins until explicitly changed.
+CURRENT V3 BASELINE SHORTCUTS: 10k / 20k / 50k / 100k / 200k
+CURRENT V3 TRANSACTION FIELD: account (V3 baseline in Demo/; not the final production data model. Phase 02 architecture is unchanged.)</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1415,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>50k / 100k / 200k / 500k</t>
+          <t>10k / 20k / 50k / 100k / 200k</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -1710,7 +1713,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>50k / 100k / 200k / 500k</t>
+          <t>10k / 20k / 50k / 100k / 200k</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -2304,6 +2307,8 @@
           <t>Dựng nền tảng code cho Tiền Đây dựa trên UX/UI v3 đã chốt.
 MỤC TIÊU
 Có architecture và data model đủ sạch để xây MVP.
+CURRENT V3 TRANSACTION FIELD: account
+(This is the V3 baseline in Demo/. It is not the final production data model. Phase 02 architecture below is unchanged.)
 DATA MODEL TỐI THIỂU
 Transaction:
 - id
@@ -2700,7 +2705,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Mục tiêu: 50k / 100k / 200k / 500k</t>
+          <t>Mục tiêu: 10k / 20k / 50k / 100k / 200k</t>
         </is>
       </c>
     </row>
@@ -2744,13 +2749,15 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Trong màn hình Thêm giao dịch, ngay dưới ô SỐ TIỀN thêm đúng 4 shortcut:
-50k   100k   200k   500k
+          <t>Trong màn hình Thêm giao dịch, ngay dưới ô SỐ TIỀN CURRENT V3 BASELINE SHORTCUTS: 10k / 20k / 50k / 100k / 200k
+Shortcut hiện có trong Demo/ (không đổi prototype):
+10k   20k   50k   100k   200k
 BEHAVIOR
+- 10k → 10.000
+- 20k → 20.000
 - 50k → 50.000
 - 100k → 100.000
 - 200k → 200.000
-- 500k → 500.000
 - Preset được chọn highlight theo style hiện tại.
 - User sửa số tiền thủ công và không còn khớp preset → bỏ highlight.
 - User nhập đúng preset bằng bàn phím → tự highlight preset.

</xml_diff>